<commit_message>
audit: limpia ledger y organiza handoffs
</commit_message>
<xml_diff>
--- a/shared/ajustes_cargo.xlsx
+++ b/shared/ajustes_cargo.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -728,7 +728,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Exonerado por la directiva 01/08/2026 (Carmen Ingaruca Julca). SOLO REGISTRO: el efecto ya lo hizo el AJUSTE del ledger — esta fila es para el backfill del libro_mayor.</t>
+          <t>Exonerado por la directiva 01/08/2026 (Carmen Ingaruca Julca). SOLO REGISTRO: pendiente de aplicar después de la reimputación.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -947,6 +947,126 @@
         </is>
       </c>
       <c r="J13" t="inlineStr">
+        <is>
+          <t>EXONERACION</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MULTA</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>50</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Se condona la multa de reunión: la secretaria reconoce confusión al anotar la asistencia y lo da por asistido. SOLO REGISTRO: pendiente de aplicar después de la reimputación.</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>seguimiento_pueblo|notas_2026-07|C-19-MULTA</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>EXONERACION</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MULTA</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>30</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Multa de faena/reunión condonada por indicación directa. SOLO REGISTRO: pendiente de aplicar después de la reimputación.</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>seguimiento_pueblo|notas_2026-07|F1-10-MULTA</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>EXONERACION</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>MULTA</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>12</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Asistió a faena; se condona solo el saldo pendiente de S/12 y se conserva el pago real de S/8. SOLO REGISTRO: pendiente de aplicar después de la reimputación.</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>seguimiento_pueblo|notas_2026-07|R-5-MULTA</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
         <is>
           <t>EXONERACION</t>
         </is>

</xml_diff>